<commit_message>
Email Setup updated Userinfo excel
</commit_message>
<xml_diff>
--- a/DataSource/UserInfo.xlsx
+++ b/DataSource/UserInfo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahthati\eclipse-workspace_week5_api\usermanagement\src\test\resource\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahthati\Documents\APIAutomation\WebAndAPI\DataSource\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD997335-F58F-483B-B1CB-792112732DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21E67493-DF98-4713-B708-8093F66993B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -581,7 +581,7 @@
         <v>12</v>
       </c>
       <c r="C13">
-        <v>200</v>
+        <v>404</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>